<commit_message>
Added a QCOM valuation
</commit_message>
<xml_diff>
--- a/ADBE.xlsx
+++ b/ADBE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A1671C-9EE2-984B-BCD3-DF606CCA9C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15BAD06-5B19-1C45-BC2B-42CF339A6519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="5" activeTab="15" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C15" s="20">
         <f>C3*'Statement Q'!N116</f>
-        <v>87957.6</v>
+        <v>87082.400000000009</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.2">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="C18" s="20">
         <f>C15+C17-C16</f>
-        <v>88976.6</v>
+        <v>88101.400000000009</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C19" s="91">
         <f>C16/'Statement Q'!J116</f>
-        <v>13.99502487562189</v>
+        <v>14.135678391959798</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="C34" s="20">
         <f>'Statement Q'!N116</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="C35" s="157">
         <f>C33/C34</f>
-        <v>2.4875621890547263E-3</v>
+        <v>2.5125628140703518E-3</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="C5" s="130">
         <f>'Statement Q'!N116</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="C7" s="145">
         <f>C5*C6</f>
-        <v>87957.6</v>
+        <v>87082.400000000009</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="C16" s="146">
         <f>C8/(C8+C7)</f>
-        <v>7.024119844486304E-2</v>
+        <v>7.0897090925385736E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C17" s="146">
         <f>C7/(C8+C7)</f>
-        <v>0.92975880155513702</v>
+        <v>0.92910290907461424</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="C20" s="146">
         <f>(C17*C19)+(C16*C18)</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="L8" s="131">
         <f>L7*(1+C14)/(C15-C14)</f>
-        <v>148659.76545752934</v>
+        <v>148736.69304427112</v>
       </c>
       <c r="N8" s="89"/>
       <c r="O8" s="7"/>
@@ -4734,23 +4734,23 @@
       <c r="G10" s="148"/>
       <c r="H10" s="131">
         <f>H7/(1+$C$15)^H9</f>
-        <v>7288.9293754717046</v>
+        <v>7289.2191301738449</v>
       </c>
       <c r="I10" s="131">
         <f t="shared" ref="I10:L10" si="0">I7/(1+$C$15)^I9</f>
-        <v>7542.698605632313</v>
+        <v>7543.2983029858324</v>
       </c>
       <c r="J10" s="131">
         <f t="shared" si="0"/>
-        <v>7590.379566469991</v>
+        <v>7591.2848169484878</v>
       </c>
       <c r="K10" s="131">
         <f t="shared" si="0"/>
-        <v>7555.7593812742616</v>
+        <v>7556.9609005902312</v>
       </c>
       <c r="L10" s="131">
         <f t="shared" si="0"/>
-        <v>7515.4210576381238</v>
+        <v>7516.9149682098905</v>
       </c>
       <c r="N10" s="89"/>
     </row>
@@ -4769,7 +4769,7 @@
       <c r="K11" s="128"/>
       <c r="L11" s="131">
         <f>L8/(1+C15)^L9</f>
-        <v>90268.583379384567</v>
+        <v>90333.247854782254</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C15" s="147">
         <f>WACC!C20</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="C19" s="102">
         <f>SUM(H10:L10)</f>
-        <v>37493.187986486395</v>
+        <v>37497.678118908283</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="C20" s="102">
         <f>L11</f>
-        <v>90268.583379384567</v>
+        <v>90333.247854782254</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="C21" s="107">
         <f>C19+C20</f>
-        <v>127761.77136587095</v>
+        <v>127830.92597369054</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="C24" s="107">
         <f>C21+C22-C23</f>
-        <v>126742.77136587095</v>
+        <v>126811.92597369052</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="C25" s="102">
         <f>'Statement Q'!N116</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="C26" s="150">
         <f>C24/C25</f>
-        <v>315.28052578574864</v>
+        <v>318.62292958213698</v>
       </c>
     </row>
   </sheetData>
@@ -5867,7 +5867,7 @@
       </c>
       <c r="C39" s="136">
         <f>WACC!C20</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="C44" s="150">
         <f>C43/(1+C48)^5</f>
-        <v>590.20914466880004</v>
+        <v>590.32646606357116</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C48" s="136">
         <f>WACC!C20</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="C52" s="150">
         <f>C51/(1+C48)^5</f>
-        <v>584.13935905348831</v>
+        <v>584.25547390017255</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
@@ -5994,7 +5994,7 @@
       </c>
       <c r="C56" s="136">
         <f>WACC!C20</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="C61" s="150">
         <f>C60/(1+C56)^5</f>
-        <v>551.28493570955231</v>
+        <v>551.39451977506189</v>
       </c>
     </row>
   </sheetData>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="C5" s="165">
         <f>DCF!C26</f>
-        <v>315.28052578574864</v>
+        <v>318.62292958213698</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C6" s="165">
         <f>Multiples!C44</f>
-        <v>590.20914466880004</v>
+        <v>590.32646606357116</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="C7" s="165">
         <f>Multiples!C52</f>
-        <v>584.13935905348831</v>
+        <v>584.25547390017255</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="C8" s="165">
         <f>Multiples!C61</f>
-        <v>551.28493570955231</v>
+        <v>551.39451977506189</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -6135,7 +6135,7 @@
       </c>
       <c r="C9" s="150">
         <f>AVERAGE(C5:C8)</f>
-        <v>510.22849130439738</v>
+        <v>511.14984733023562</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="C11" s="87">
         <f>(C9-C10)/C10</f>
-        <v>1.3319400882285071</v>
+        <v>1.3361510389864515</v>
       </c>
     </row>
   </sheetData>
@@ -6385,7 +6385,7 @@
       <c r="K8" s="128"/>
       <c r="L8" s="131">
         <f>L7*(1+C20)/(C21-C20)</f>
-        <v>93392.121267046983</v>
+        <v>93435.355544992402</v>
       </c>
       <c r="N8" s="89"/>
       <c r="O8" s="7"/>
@@ -6439,23 +6439,23 @@
       <c r="G10" s="148"/>
       <c r="H10" s="131">
         <f>H7/(1+$C$21)^H9</f>
-        <v>7633.7140791749825</v>
+        <v>7634.0175400037679</v>
       </c>
       <c r="I10" s="131">
         <f t="shared" ref="I10:L10" si="1">I7/(1+$C$21)^I9</f>
-        <v>6977.918616026097</v>
+        <v>6978.473409415823</v>
       </c>
       <c r="J10" s="131">
         <f t="shared" si="1"/>
-        <v>6378.4610881242106</v>
+        <v>6379.2218017224604</v>
       </c>
       <c r="K10" s="131">
         <f t="shared" si="1"/>
-        <v>5830.501628275586</v>
+        <v>5831.4287965421563</v>
       </c>
       <c r="L10" s="131">
         <f t="shared" si="1"/>
-        <v>5329.616151553807</v>
+        <v>5330.6755692299694</v>
       </c>
       <c r="N10" s="89"/>
     </row>
@@ -6474,7 +6474,7 @@
       <c r="K11" s="128"/>
       <c r="L11" s="131">
         <f>L8/(1+C21)^L9</f>
-        <v>56709.187315249066</v>
+        <v>56746.717693483079</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -6499,7 +6499,7 @@
       </c>
       <c r="C16" s="196">
         <f>C36</f>
-        <v>218.50845492140238</v>
+        <v>220.80787640803328</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="C21" s="201">
         <f>WACC!C20</f>
-        <v>0.10492134463407983</v>
+        <v>0.104877422761327</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="C22" s="202">
         <f>'Statement Q'!N116</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.2">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="C23" s="202">
         <f>C15*C22</f>
-        <v>87957.6</v>
+        <v>87082.400000000009</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C26" s="203">
         <f>C23+C25-C24</f>
-        <v>88976.6</v>
+        <v>88101.400000000009</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -6599,7 +6599,7 @@
       </c>
       <c r="C29" s="202">
         <f>SUM(H10:L10)</f>
-        <v>32150.211563154684</v>
+        <v>32153.817116914179</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C30" s="202">
         <f>L11</f>
-        <v>56709.187315249066</v>
+        <v>56746.717693483079</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="C31" s="205">
         <f>C29+C30</f>
-        <v>88859.39887840375</v>
+        <v>88900.53481039725</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="C34" s="205">
         <f>C31+C32-C33</f>
-        <v>87840.39887840375</v>
+        <v>87881.53481039725</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="C35" s="202">
         <f>C22</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="36" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="C36" s="208">
         <f>C34/C35</f>
-        <v>218.50845492140238</v>
+        <v>220.80787640803328</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -7109,17 +7109,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -17535,14 +17535,14 @@
         <v>404</v>
       </c>
       <c r="J116" s="27">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="K116" s="20"/>
       <c r="L116" s="20"/>
       <c r="M116" s="20"/>
       <c r="N116" s="20">
         <f>J116</f>
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="117" spans="1:19" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -29109,12 +29109,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -29122,6 +29116,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>